<commit_message>
EGGRA, GDPBES< FOICStCT, ERWD extend to 2070
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/EGGRA/Exogenous GDP Growth Rate Adjustment.xlsx
+++ b/InputData/ctrl-settings/EGGRA/Exogenous GDP Growth Rate Adjustment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeff Rissman\CodeRepositories\eps-us\InputData\ctrl-settings\EGGRA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\ctrl-settings\EGGRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D77B80-46D1-401E-A779-175C6F49CDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D1F1EB-3C55-43B4-ADAC-9B35B75B77D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9555" yWindow="345" windowWidth="22590" windowHeight="21675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -201,7 +201,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -211,7 +211,6 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -497,155 +496,155 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="52.5703125" customWidth="1"/>
+    <col min="2" max="2" width="52.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" s="1"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B6" s="6"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B8" s="3"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A14" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A15" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A17" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A19" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A20" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A21" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A22" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A23" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A25" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A26" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A27" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A29" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B29" s="2"/>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A30" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A31" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A32" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.75">
       <c r="A33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.75">
       <c r="A34" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.75">
       <c r="A35" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.75">
       <c r="A36" t="s">
         <v>24</v>
       </c>
@@ -661,13 +660,13 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AZ2"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="51.140625" customWidth="1"/>
+    <col min="1" max="1" width="51.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -764,8 +763,68 @@
       <c r="AF1">
         <v>2050</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG1">
+        <v>2051</v>
+      </c>
+      <c r="AH1">
+        <v>2052</v>
+      </c>
+      <c r="AI1">
+        <v>2053</v>
+      </c>
+      <c r="AJ1">
+        <v>2054</v>
+      </c>
+      <c r="AK1">
+        <v>2055</v>
+      </c>
+      <c r="AL1">
+        <v>2056</v>
+      </c>
+      <c r="AM1">
+        <v>2057</v>
+      </c>
+      <c r="AN1">
+        <v>2058</v>
+      </c>
+      <c r="AO1">
+        <v>2059</v>
+      </c>
+      <c r="AP1">
+        <v>2060</v>
+      </c>
+      <c r="AQ1">
+        <v>2061</v>
+      </c>
+      <c r="AR1">
+        <v>2062</v>
+      </c>
+      <c r="AS1">
+        <v>2063</v>
+      </c>
+      <c r="AT1">
+        <v>2064</v>
+      </c>
+      <c r="AU1">
+        <v>2065</v>
+      </c>
+      <c r="AV1">
+        <v>2066</v>
+      </c>
+      <c r="AW1">
+        <v>2067</v>
+      </c>
+      <c r="AX1">
+        <v>2068</v>
+      </c>
+      <c r="AY1">
+        <v>2069</v>
+      </c>
+      <c r="AZ1">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="2" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -860,6 +919,66 @@
         <v>0</v>
       </c>
       <c r="AF2">
+        <v>0</v>
+      </c>
+      <c r="AG2">
+        <v>0</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
+        <v>0</v>
+      </c>
+      <c r="AK2">
+        <v>0</v>
+      </c>
+      <c r="AL2">
+        <v>0</v>
+      </c>
+      <c r="AM2">
+        <v>0</v>
+      </c>
+      <c r="AN2">
+        <v>0</v>
+      </c>
+      <c r="AO2">
+        <v>0</v>
+      </c>
+      <c r="AP2">
+        <v>0</v>
+      </c>
+      <c r="AQ2">
+        <v>0</v>
+      </c>
+      <c r="AR2">
+        <v>0</v>
+      </c>
+      <c r="AS2">
+        <v>0</v>
+      </c>
+      <c r="AT2">
+        <v>0</v>
+      </c>
+      <c r="AU2">
+        <v>0</v>
+      </c>
+      <c r="AV2">
+        <v>0</v>
+      </c>
+      <c r="AW2">
+        <v>0</v>
+      </c>
+      <c r="AX2">
+        <v>0</v>
+      </c>
+      <c r="AY2">
+        <v>0</v>
+      </c>
+      <c r="AZ2">
         <v>0</v>
       </c>
     </row>
@@ -875,26 +994,26 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="43.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="1" max="1" width="43.1328125" customWidth="1"/>
+    <col min="2" max="2" width="10.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>32</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>